<commit_message>
finished final data cleaning, feature engineering
</commit_message>
<xml_diff>
--- a/Dataset/FeatureTable.xlsx
+++ b/Dataset/FeatureTable.xlsx
@@ -303,7 +303,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -314,12 +314,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -371,22 +365,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -696,35 +684,35 @@
   <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="16.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="44.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="14.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="16.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="44.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="14.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
-      <c r="A1" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25" customFormat="1" s="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -733,14 +721,14 @@
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
@@ -749,14 +737,14 @@
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="28.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="28.5" customFormat="1" s="1">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -769,14 +757,14 @@
       <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
@@ -789,14 +777,14 @@
       <c r="D5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="28.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="28.5" customFormat="1" s="1">
       <c r="A6" s="3" t="s">
         <v>21</v>
       </c>
@@ -809,14 +797,14 @@
       <c r="D6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -827,14 +815,14 @@
         <v>14</v>
       </c>
       <c r="D7" s="3"/>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>25</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="39.75" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="39.75" customFormat="1" s="1">
       <c r="A8" s="3" t="s">
         <v>26</v>
       </c>
@@ -845,14 +833,14 @@
         <v>14</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="39.75" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="39.75" customFormat="1" s="1">
       <c r="A9" s="3" t="s">
         <v>28</v>
       </c>
@@ -863,14 +851,14 @@
         <v>14</v>
       </c>
       <c r="D9" s="3"/>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="46.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A10" s="3" t="s">
         <v>30</v>
       </c>
@@ -881,14 +869,14 @@
         <v>14</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -899,14 +887,14 @@
         <v>33</v>
       </c>
       <c r="D11" s="3"/>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="46.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A12" s="3" t="s">
         <v>35</v>
       </c>
@@ -917,14 +905,14 @@
         <v>14</v>
       </c>
       <c r="D12" s="3"/>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>36</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="60" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A13" s="3" t="s">
         <v>37</v>
       </c>
@@ -935,14 +923,14 @@
         <v>14</v>
       </c>
       <c r="D13" s="3"/>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>38</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A14" s="3" t="s">
         <v>39</v>
       </c>
@@ -953,14 +941,14 @@
         <v>33</v>
       </c>
       <c r="D14" s="3"/>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>40</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A15" s="3" t="s">
         <v>41</v>
       </c>
@@ -971,14 +959,14 @@
         <v>33</v>
       </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A16" s="3" t="s">
         <v>43</v>
       </c>
@@ -989,14 +977,14 @@
         <v>33</v>
       </c>
       <c r="D16" s="3"/>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>44</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A17" s="3" t="s">
         <v>45</v>
       </c>
@@ -1007,14 +995,14 @@
         <v>33</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A18" s="3" t="s">
         <v>47</v>
       </c>
@@ -1025,14 +1013,14 @@
         <v>33</v>
       </c>
       <c r="D18" s="3"/>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A19" s="3" t="s">
         <v>49</v>
       </c>
@@ -1043,14 +1031,14 @@
         <v>33</v>
       </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>50</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A20" s="3" t="s">
         <v>51</v>
       </c>
@@ -1061,14 +1049,14 @@
         <v>14</v>
       </c>
       <c r="D20" s="3"/>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A21" s="3" t="s">
         <v>53</v>
       </c>
@@ -1079,14 +1067,14 @@
         <v>14</v>
       </c>
       <c r="D21" s="3"/>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>54</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="33" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A22" s="3" t="s">
         <v>55</v>
       </c>
@@ -1097,14 +1085,14 @@
         <v>14</v>
       </c>
       <c r="D22" s="3"/>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="28.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A23" s="3" t="s">
         <v>57</v>
       </c>
@@ -1115,14 +1103,14 @@
         <v>33</v>
       </c>
       <c r="D23" s="3"/>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>58</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="46.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A24" s="3" t="s">
         <v>59</v>
       </c>
@@ -1133,14 +1121,14 @@
         <v>14</v>
       </c>
       <c r="D24" s="3"/>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="62.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A25" s="3" t="s">
         <v>61</v>
       </c>
@@ -1151,14 +1139,14 @@
         <v>14</v>
       </c>
       <c r="D25" s="3"/>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="3" t="s">
         <v>62</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A26" s="3" t="s">
         <v>63</v>
       </c>
@@ -1169,12 +1157,12 @@
         <v>14</v>
       </c>
       <c r="D26" s="3"/>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F26" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A27" s="3" t="s">
         <v>65</v>
       </c>
@@ -1185,14 +1173,14 @@
         <v>14</v>
       </c>
       <c r="D27" s="3"/>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A28" s="3" t="s">
         <v>66</v>
       </c>
@@ -1203,14 +1191,14 @@
         <v>14</v>
       </c>
       <c r="D28" s="3"/>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A29" s="3" t="s">
         <v>67</v>
       </c>
@@ -1221,14 +1209,14 @@
         <v>14</v>
       </c>
       <c r="D29" s="3"/>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A30" s="3" t="s">
         <v>68</v>
       </c>
@@ -1239,14 +1227,14 @@
         <v>14</v>
       </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A31" s="3" t="s">
         <v>69</v>
       </c>
@@ -1257,14 +1245,14 @@
         <v>14</v>
       </c>
       <c r="D31" s="3"/>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="73.5" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A32" s="3" t="s">
         <v>70</v>
       </c>
@@ -1275,14 +1263,14 @@
         <v>14</v>
       </c>
       <c r="D32" s="3"/>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A33" s="3" t="s">
         <v>71</v>
       </c>
@@ -1293,14 +1281,14 @@
         <v>14</v>
       </c>
       <c r="D33" s="3"/>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A34" s="3" t="s">
         <v>72</v>
       </c>
@@ -1311,14 +1299,14 @@
         <v>14</v>
       </c>
       <c r="D34" s="3"/>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A35" s="3" t="s">
         <v>73</v>
       </c>
@@ -1329,14 +1317,14 @@
         <v>14</v>
       </c>
       <c r="D35" s="3"/>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A36" s="3" t="s">
         <v>74</v>
       </c>
@@ -1347,14 +1335,14 @@
         <v>14</v>
       </c>
       <c r="D36" s="3"/>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A37" s="3" t="s">
         <v>75</v>
       </c>
@@ -1365,14 +1353,14 @@
         <v>14</v>
       </c>
       <c r="D37" s="3"/>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A38" s="3" t="s">
         <v>76</v>
       </c>
@@ -1383,14 +1371,14 @@
         <v>14</v>
       </c>
       <c r="D38" s="3"/>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A39" s="3" t="s">
         <v>77</v>
       </c>
@@ -1401,14 +1389,14 @@
         <v>14</v>
       </c>
       <c r="D39" s="3"/>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A40" s="3" t="s">
         <v>78</v>
       </c>
@@ -1419,14 +1407,14 @@
         <v>14</v>
       </c>
       <c r="D40" s="3"/>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A41" s="3" t="s">
         <v>79</v>
       </c>
@@ -1437,14 +1425,14 @@
         <v>14</v>
       </c>
       <c r="D41" s="3"/>
-      <c r="E41" s="4" t="s">
+      <c r="E41" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A42" s="3" t="s">
         <v>80</v>
       </c>
@@ -1455,14 +1443,14 @@
         <v>14</v>
       </c>
       <c r="D42" s="3"/>
-      <c r="E42" s="4" t="s">
+      <c r="E42" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A43" s="3" t="s">
         <v>81</v>
       </c>
@@ -1473,14 +1461,14 @@
         <v>14</v>
       </c>
       <c r="D43" s="3"/>
-      <c r="E43" s="4" t="s">
+      <c r="E43" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A44" s="3" t="s">
         <v>82</v>
       </c>
@@ -1491,14 +1479,14 @@
         <v>14</v>
       </c>
       <c r="D44" s="3"/>
-      <c r="E44" s="4" t="s">
+      <c r="E44" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A45" s="3" t="s">
         <v>83</v>
       </c>
@@ -1509,14 +1497,14 @@
         <v>14</v>
       </c>
       <c r="D45" s="3"/>
-      <c r="E45" s="4" t="s">
+      <c r="E45" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A46" s="3" t="s">
         <v>84</v>
       </c>
@@ -1527,14 +1515,14 @@
         <v>14</v>
       </c>
       <c r="D46" s="3"/>
-      <c r="E46" s="4" t="s">
+      <c r="E46" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A47" s="3" t="s">
         <v>85</v>
       </c>
@@ -1545,14 +1533,14 @@
         <v>14</v>
       </c>
       <c r="D47" s="3"/>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A48" s="3" t="s">
         <v>86</v>
       </c>
@@ -1563,14 +1551,14 @@
         <v>14</v>
       </c>
       <c r="D48" s="3"/>
-      <c r="E48" s="4" t="s">
+      <c r="E48" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A49" s="3" t="s">
         <v>87</v>
       </c>
@@ -1581,14 +1569,14 @@
         <v>14</v>
       </c>
       <c r="D49" s="3"/>
-      <c r="E49" s="4" t="s">
+      <c r="E49" s="3" t="s">
         <v>88</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A50" s="3" t="s">
         <v>89</v>
       </c>
@@ -1599,14 +1587,14 @@
         <v>14</v>
       </c>
       <c r="D50" s="3"/>
-      <c r="E50" s="4" t="s">
+      <c r="E50" s="3" t="s">
         <v>90</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="17.25" customFormat="1" s="2">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A51" s="3" t="s">
         <v>91</v>
       </c>
@@ -1617,7 +1605,7 @@
         <v>14</v>
       </c>
       <c r="D51" s="3"/>
-      <c r="E51" s="4" t="s">
+      <c r="E51" s="3" t="s">
         <v>93</v>
       </c>
       <c r="F51" s="3" t="s">

</xml_diff>